<commit_message>
Add HRMS state master GST mapping
</commit_message>
<xml_diff>
--- a/mock-db/hrms_mock_database.xlsx
+++ b/mock-db/hrms_mock_database.xlsx
@@ -9,6 +9,7 @@
     <sheet name="attendance" sheetId="4" r:id="rId4"/>
     <sheet name="keyholders" sheetId="5" r:id="rId5"/>
     <sheet name="module_rows" sheetId="6" r:id="rId6"/>
+    <sheet name="state_masters" sheetId="7" r:id="rId7"/>
   </sheets>
 </workbook>
 </file>
@@ -623,4 +624,661 @@
     <ignoredError numberStoredAsText="1" sqref="A1:C1"/>
   </ignoredErrors>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:E38"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="str">
+        <v>state_code</v>
+      </c>
+      <c r="B1" t="str">
+        <v>state_name</v>
+      </c>
+      <c r="C1" t="str">
+        <v>gst_state_code</v>
+      </c>
+      <c r="D1" t="str">
+        <v>country</v>
+      </c>
+      <c r="E1" t="str">
+        <v>status</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="str">
+        <v>01</v>
+      </c>
+      <c r="B2" t="str">
+        <v>Jammu and Kashmir</v>
+      </c>
+      <c r="C2" t="str">
+        <v>01</v>
+      </c>
+      <c r="D2" t="str">
+        <v>India</v>
+      </c>
+      <c r="E2" t="str">
+        <v>Active</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="str">
+        <v>02</v>
+      </c>
+      <c r="B3" t="str">
+        <v>Himachal Pradesh</v>
+      </c>
+      <c r="C3" t="str">
+        <v>02</v>
+      </c>
+      <c r="D3" t="str">
+        <v>India</v>
+      </c>
+      <c r="E3" t="str">
+        <v>Active</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="str">
+        <v>03</v>
+      </c>
+      <c r="B4" t="str">
+        <v>Punjab</v>
+      </c>
+      <c r="C4" t="str">
+        <v>03</v>
+      </c>
+      <c r="D4" t="str">
+        <v>India</v>
+      </c>
+      <c r="E4" t="str">
+        <v>Active</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="str">
+        <v>04</v>
+      </c>
+      <c r="B5" t="str">
+        <v>Chandigarh</v>
+      </c>
+      <c r="C5" t="str">
+        <v>04</v>
+      </c>
+      <c r="D5" t="str">
+        <v>India</v>
+      </c>
+      <c r="E5" t="str">
+        <v>Active</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="str">
+        <v>05</v>
+      </c>
+      <c r="B6" t="str">
+        <v>Uttarakhand</v>
+      </c>
+      <c r="C6" t="str">
+        <v>05</v>
+      </c>
+      <c r="D6" t="str">
+        <v>India</v>
+      </c>
+      <c r="E6" t="str">
+        <v>Active</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="str">
+        <v>06</v>
+      </c>
+      <c r="B7" t="str">
+        <v>Haryana</v>
+      </c>
+      <c r="C7" t="str">
+        <v>06</v>
+      </c>
+      <c r="D7" t="str">
+        <v>India</v>
+      </c>
+      <c r="E7" t="str">
+        <v>Active</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="str">
+        <v>07</v>
+      </c>
+      <c r="B8" t="str">
+        <v>Delhi</v>
+      </c>
+      <c r="C8" t="str">
+        <v>07</v>
+      </c>
+      <c r="D8" t="str">
+        <v>India</v>
+      </c>
+      <c r="E8" t="str">
+        <v>Active</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="str">
+        <v>08</v>
+      </c>
+      <c r="B9" t="str">
+        <v>Rajasthan</v>
+      </c>
+      <c r="C9" t="str">
+        <v>08</v>
+      </c>
+      <c r="D9" t="str">
+        <v>India</v>
+      </c>
+      <c r="E9" t="str">
+        <v>Active</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="str">
+        <v>09</v>
+      </c>
+      <c r="B10" t="str">
+        <v>Uttar Pradesh</v>
+      </c>
+      <c r="C10" t="str">
+        <v>09</v>
+      </c>
+      <c r="D10" t="str">
+        <v>India</v>
+      </c>
+      <c r="E10" t="str">
+        <v>Active</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="str">
+        <v>10</v>
+      </c>
+      <c r="B11" t="str">
+        <v>Bihar</v>
+      </c>
+      <c r="C11" t="str">
+        <v>10</v>
+      </c>
+      <c r="D11" t="str">
+        <v>India</v>
+      </c>
+      <c r="E11" t="str">
+        <v>Active</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="str">
+        <v>11</v>
+      </c>
+      <c r="B12" t="str">
+        <v>Sikkim</v>
+      </c>
+      <c r="C12" t="str">
+        <v>11</v>
+      </c>
+      <c r="D12" t="str">
+        <v>India</v>
+      </c>
+      <c r="E12" t="str">
+        <v>Active</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="str">
+        <v>12</v>
+      </c>
+      <c r="B13" t="str">
+        <v>Arunachal Pradesh</v>
+      </c>
+      <c r="C13" t="str">
+        <v>12</v>
+      </c>
+      <c r="D13" t="str">
+        <v>India</v>
+      </c>
+      <c r="E13" t="str">
+        <v>Active</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="str">
+        <v>13</v>
+      </c>
+      <c r="B14" t="str">
+        <v>Nagaland</v>
+      </c>
+      <c r="C14" t="str">
+        <v>13</v>
+      </c>
+      <c r="D14" t="str">
+        <v>India</v>
+      </c>
+      <c r="E14" t="str">
+        <v>Active</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="str">
+        <v>14</v>
+      </c>
+      <c r="B15" t="str">
+        <v>Manipur</v>
+      </c>
+      <c r="C15" t="str">
+        <v>14</v>
+      </c>
+      <c r="D15" t="str">
+        <v>India</v>
+      </c>
+      <c r="E15" t="str">
+        <v>Active</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="str">
+        <v>15</v>
+      </c>
+      <c r="B16" t="str">
+        <v>Mizoram</v>
+      </c>
+      <c r="C16" t="str">
+        <v>15</v>
+      </c>
+      <c r="D16" t="str">
+        <v>India</v>
+      </c>
+      <c r="E16" t="str">
+        <v>Active</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="str">
+        <v>16</v>
+      </c>
+      <c r="B17" t="str">
+        <v>Tripura</v>
+      </c>
+      <c r="C17" t="str">
+        <v>16</v>
+      </c>
+      <c r="D17" t="str">
+        <v>India</v>
+      </c>
+      <c r="E17" t="str">
+        <v>Active</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="str">
+        <v>17</v>
+      </c>
+      <c r="B18" t="str">
+        <v>Meghalaya</v>
+      </c>
+      <c r="C18" t="str">
+        <v>17</v>
+      </c>
+      <c r="D18" t="str">
+        <v>India</v>
+      </c>
+      <c r="E18" t="str">
+        <v>Active</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="str">
+        <v>18</v>
+      </c>
+      <c r="B19" t="str">
+        <v>Assam</v>
+      </c>
+      <c r="C19" t="str">
+        <v>18</v>
+      </c>
+      <c r="D19" t="str">
+        <v>India</v>
+      </c>
+      <c r="E19" t="str">
+        <v>Active</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="str">
+        <v>19</v>
+      </c>
+      <c r="B20" t="str">
+        <v>West Bengal</v>
+      </c>
+      <c r="C20" t="str">
+        <v>19</v>
+      </c>
+      <c r="D20" t="str">
+        <v>India</v>
+      </c>
+      <c r="E20" t="str">
+        <v>Active</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="str">
+        <v>20</v>
+      </c>
+      <c r="B21" t="str">
+        <v>Jharkhand</v>
+      </c>
+      <c r="C21" t="str">
+        <v>20</v>
+      </c>
+      <c r="D21" t="str">
+        <v>India</v>
+      </c>
+      <c r="E21" t="str">
+        <v>Active</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="str">
+        <v>21</v>
+      </c>
+      <c r="B22" t="str">
+        <v>Odisha</v>
+      </c>
+      <c r="C22" t="str">
+        <v>21</v>
+      </c>
+      <c r="D22" t="str">
+        <v>India</v>
+      </c>
+      <c r="E22" t="str">
+        <v>Active</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="str">
+        <v>22</v>
+      </c>
+      <c r="B23" t="str">
+        <v>Chhattisgarh</v>
+      </c>
+      <c r="C23" t="str">
+        <v>22</v>
+      </c>
+      <c r="D23" t="str">
+        <v>India</v>
+      </c>
+      <c r="E23" t="str">
+        <v>Active</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="str">
+        <v>23</v>
+      </c>
+      <c r="B24" t="str">
+        <v>Madhya Pradesh</v>
+      </c>
+      <c r="C24" t="str">
+        <v>23</v>
+      </c>
+      <c r="D24" t="str">
+        <v>India</v>
+      </c>
+      <c r="E24" t="str">
+        <v>Active</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="str">
+        <v>24</v>
+      </c>
+      <c r="B25" t="str">
+        <v>Gujarat</v>
+      </c>
+      <c r="C25" t="str">
+        <v>24</v>
+      </c>
+      <c r="D25" t="str">
+        <v>India</v>
+      </c>
+      <c r="E25" t="str">
+        <v>Active</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="str">
+        <v>26</v>
+      </c>
+      <c r="B26" t="str">
+        <v>Dadra and Nagar Haveli and Daman and Diu</v>
+      </c>
+      <c r="C26" t="str">
+        <v>26</v>
+      </c>
+      <c r="D26" t="str">
+        <v>India</v>
+      </c>
+      <c r="E26" t="str">
+        <v>Active</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="str">
+        <v>27</v>
+      </c>
+      <c r="B27" t="str">
+        <v>Maharashtra</v>
+      </c>
+      <c r="C27" t="str">
+        <v>27</v>
+      </c>
+      <c r="D27" t="str">
+        <v>India</v>
+      </c>
+      <c r="E27" t="str">
+        <v>Active</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="str">
+        <v>29</v>
+      </c>
+      <c r="B28" t="str">
+        <v>Karnataka</v>
+      </c>
+      <c r="C28" t="str">
+        <v>29</v>
+      </c>
+      <c r="D28" t="str">
+        <v>India</v>
+      </c>
+      <c r="E28" t="str">
+        <v>Active</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="str">
+        <v>30</v>
+      </c>
+      <c r="B29" t="str">
+        <v>Goa</v>
+      </c>
+      <c r="C29" t="str">
+        <v>30</v>
+      </c>
+      <c r="D29" t="str">
+        <v>India</v>
+      </c>
+      <c r="E29" t="str">
+        <v>Active</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="str">
+        <v>31</v>
+      </c>
+      <c r="B30" t="str">
+        <v>Lakshadweep</v>
+      </c>
+      <c r="C30" t="str">
+        <v>31</v>
+      </c>
+      <c r="D30" t="str">
+        <v>India</v>
+      </c>
+      <c r="E30" t="str">
+        <v>Active</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="str">
+        <v>32</v>
+      </c>
+      <c r="B31" t="str">
+        <v>Kerala</v>
+      </c>
+      <c r="C31" t="str">
+        <v>32</v>
+      </c>
+      <c r="D31" t="str">
+        <v>India</v>
+      </c>
+      <c r="E31" t="str">
+        <v>Active</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="str">
+        <v>33</v>
+      </c>
+      <c r="B32" t="str">
+        <v>Tamil Nadu</v>
+      </c>
+      <c r="C32" t="str">
+        <v>33</v>
+      </c>
+      <c r="D32" t="str">
+        <v>India</v>
+      </c>
+      <c r="E32" t="str">
+        <v>Active</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="str">
+        <v>34</v>
+      </c>
+      <c r="B33" t="str">
+        <v>Puducherry</v>
+      </c>
+      <c r="C33" t="str">
+        <v>34</v>
+      </c>
+      <c r="D33" t="str">
+        <v>India</v>
+      </c>
+      <c r="E33" t="str">
+        <v>Active</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="str">
+        <v>35</v>
+      </c>
+      <c r="B34" t="str">
+        <v>Andaman and Nicobar Islands</v>
+      </c>
+      <c r="C34" t="str">
+        <v>35</v>
+      </c>
+      <c r="D34" t="str">
+        <v>India</v>
+      </c>
+      <c r="E34" t="str">
+        <v>Active</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="str">
+        <v>36</v>
+      </c>
+      <c r="B35" t="str">
+        <v>Telangana</v>
+      </c>
+      <c r="C35" t="str">
+        <v>36</v>
+      </c>
+      <c r="D35" t="str">
+        <v>India</v>
+      </c>
+      <c r="E35" t="str">
+        <v>Active</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="str">
+        <v>37</v>
+      </c>
+      <c r="B36" t="str">
+        <v>Andhra Pradesh</v>
+      </c>
+      <c r="C36" t="str">
+        <v>37</v>
+      </c>
+      <c r="D36" t="str">
+        <v>India</v>
+      </c>
+      <c r="E36" t="str">
+        <v>Active</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="str">
+        <v>38</v>
+      </c>
+      <c r="B37" t="str">
+        <v>Ladakh</v>
+      </c>
+      <c r="C37" t="str">
+        <v>38</v>
+      </c>
+      <c r="D37" t="str">
+        <v>India</v>
+      </c>
+      <c r="E37" t="str">
+        <v>Active</v>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="str">
+        <v>97</v>
+      </c>
+      <c r="B38" t="str">
+        <v>Other Territory</v>
+      </c>
+      <c r="C38" t="str">
+        <v>97</v>
+      </c>
+      <c r="D38" t="str">
+        <v>India</v>
+      </c>
+      <c r="E38" t="str">
+        <v>Active</v>
+      </c>
+    </row>
+  </sheetData>
+  <ignoredErrors>
+    <ignoredError numberStoredAsText="1" sqref="A1:E38"/>
+  </ignoredErrors>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Add HRMS pincode city state mapping
</commit_message>
<xml_diff>
--- a/mock-db/hrms_mock_database.xlsx
+++ b/mock-db/hrms_mock_database.xlsx
@@ -10,6 +10,7 @@
     <sheet name="keyholders" sheetId="5" r:id="rId5"/>
     <sheet name="module_rows" sheetId="6" r:id="rId6"/>
     <sheet name="state_masters" sheetId="7" r:id="rId7"/>
+    <sheet name="pincode_masters" sheetId="8" r:id="rId8"/>
   </sheets>
 </workbook>
 </file>
@@ -1281,4 +1282,155 @@
     <ignoredError numberStoredAsText="1" sqref="A1:E38"/>
   </ignoredErrors>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:F7"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="str">
+        <v>pincode</v>
+      </c>
+      <c r="B1" t="str">
+        <v>city</v>
+      </c>
+      <c r="C1" t="str">
+        <v>state_name</v>
+      </c>
+      <c r="D1" t="str">
+        <v>gst_state_code</v>
+      </c>
+      <c r="E1" t="str">
+        <v>country</v>
+      </c>
+      <c r="F1" t="str">
+        <v>status</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="str">
+        <v>700029</v>
+      </c>
+      <c r="B2" t="str">
+        <v>Kolkata</v>
+      </c>
+      <c r="C2" t="str">
+        <v>West Bengal</v>
+      </c>
+      <c r="D2" t="str">
+        <v>19</v>
+      </c>
+      <c r="E2" t="str">
+        <v>India</v>
+      </c>
+      <c r="F2" t="str">
+        <v>Active</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="str">
+        <v>700045</v>
+      </c>
+      <c r="B3" t="str">
+        <v>Kolkata</v>
+      </c>
+      <c r="C3" t="str">
+        <v>West Bengal</v>
+      </c>
+      <c r="D3" t="str">
+        <v>19</v>
+      </c>
+      <c r="E3" t="str">
+        <v>India</v>
+      </c>
+      <c r="F3" t="str">
+        <v>Active</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="str">
+        <v>700091</v>
+      </c>
+      <c r="B4" t="str">
+        <v>Kolkata</v>
+      </c>
+      <c r="C4" t="str">
+        <v>West Bengal</v>
+      </c>
+      <c r="D4" t="str">
+        <v>19</v>
+      </c>
+      <c r="E4" t="str">
+        <v>India</v>
+      </c>
+      <c r="F4" t="str">
+        <v>Active</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="str">
+        <v>700135</v>
+      </c>
+      <c r="B5" t="str">
+        <v>Rajarhat</v>
+      </c>
+      <c r="C5" t="str">
+        <v>West Bengal</v>
+      </c>
+      <c r="D5" t="str">
+        <v>19</v>
+      </c>
+      <c r="E5" t="str">
+        <v>India</v>
+      </c>
+      <c r="F5" t="str">
+        <v>Active</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="str">
+        <v>700156</v>
+      </c>
+      <c r="B6" t="str">
+        <v>Newtown</v>
+      </c>
+      <c r="C6" t="str">
+        <v>West Bengal</v>
+      </c>
+      <c r="D6" t="str">
+        <v>19</v>
+      </c>
+      <c r="E6" t="str">
+        <v>India</v>
+      </c>
+      <c r="F6" t="str">
+        <v>Active</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="str">
+        <v>700157</v>
+      </c>
+      <c r="B7" t="str">
+        <v>Rajarhat</v>
+      </c>
+      <c r="C7" t="str">
+        <v>West Bengal</v>
+      </c>
+      <c r="D7" t="str">
+        <v>19</v>
+      </c>
+      <c r="E7" t="str">
+        <v>India</v>
+      </c>
+      <c r="F7" t="str">
+        <v>Active</v>
+      </c>
+    </row>
+  </sheetData>
+  <ignoredErrors>
+    <ignoredError numberStoredAsText="1" sqref="A1:F7"/>
+  </ignoredErrors>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Add HRMS West Bengal city master
</commit_message>
<xml_diff>
--- a/mock-db/hrms_mock_database.xlsx
+++ b/mock-db/hrms_mock_database.xlsx
@@ -11,6 +11,7 @@
     <sheet name="module_rows" sheetId="6" r:id="rId6"/>
     <sheet name="state_masters" sheetId="7" r:id="rId7"/>
     <sheet name="pincode_masters" sheetId="8" r:id="rId8"/>
+    <sheet name="city_masters" sheetId="9" r:id="rId9"/>
   </sheets>
 </workbook>
 </file>
@@ -1433,4 +1434,843 @@
     <ignoredError numberStoredAsText="1" sqref="A1:F7"/>
   </ignoredErrors>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:G36"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="str">
+        <v>city_id</v>
+      </c>
+      <c r="B1" t="str">
+        <v>city</v>
+      </c>
+      <c r="C1" t="str">
+        <v>district</v>
+      </c>
+      <c r="D1" t="str">
+        <v>state_name</v>
+      </c>
+      <c r="E1" t="str">
+        <v>gst_state_code</v>
+      </c>
+      <c r="F1" t="str">
+        <v>country</v>
+      </c>
+      <c r="G1" t="str">
+        <v>status</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="str">
+        <v>WB-ALIPURDUAR</v>
+      </c>
+      <c r="B2" t="str">
+        <v>Alipurduar</v>
+      </c>
+      <c r="C2" t="str">
+        <v>Alipurduar</v>
+      </c>
+      <c r="D2" t="str">
+        <v>West Bengal</v>
+      </c>
+      <c r="E2" t="str">
+        <v>19</v>
+      </c>
+      <c r="F2" t="str">
+        <v>India</v>
+      </c>
+      <c r="G2" t="str">
+        <v>Active</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="str">
+        <v>WB-ASANSOL</v>
+      </c>
+      <c r="B3" t="str">
+        <v>Asansol</v>
+      </c>
+      <c r="C3" t="str">
+        <v>Paschim Bardhaman</v>
+      </c>
+      <c r="D3" t="str">
+        <v>West Bengal</v>
+      </c>
+      <c r="E3" t="str">
+        <v>19</v>
+      </c>
+      <c r="F3" t="str">
+        <v>India</v>
+      </c>
+      <c r="G3" t="str">
+        <v>Active</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="str">
+        <v>WB-BAHARAMPUR</v>
+      </c>
+      <c r="B4" t="str">
+        <v>Baharampur</v>
+      </c>
+      <c r="C4" t="str">
+        <v>Murshidabad</v>
+      </c>
+      <c r="D4" t="str">
+        <v>West Bengal</v>
+      </c>
+      <c r="E4" t="str">
+        <v>19</v>
+      </c>
+      <c r="F4" t="str">
+        <v>India</v>
+      </c>
+      <c r="G4" t="str">
+        <v>Active</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="str">
+        <v>WB-BALURGHAT</v>
+      </c>
+      <c r="B5" t="str">
+        <v>Balurghat</v>
+      </c>
+      <c r="C5" t="str">
+        <v>Dakshin Dinajpur</v>
+      </c>
+      <c r="D5" t="str">
+        <v>West Bengal</v>
+      </c>
+      <c r="E5" t="str">
+        <v>19</v>
+      </c>
+      <c r="F5" t="str">
+        <v>India</v>
+      </c>
+      <c r="G5" t="str">
+        <v>Active</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="str">
+        <v>WB-BANKURA</v>
+      </c>
+      <c r="B6" t="str">
+        <v>Bankura</v>
+      </c>
+      <c r="C6" t="str">
+        <v>Bankura</v>
+      </c>
+      <c r="D6" t="str">
+        <v>West Bengal</v>
+      </c>
+      <c r="E6" t="str">
+        <v>19</v>
+      </c>
+      <c r="F6" t="str">
+        <v>India</v>
+      </c>
+      <c r="G6" t="str">
+        <v>Active</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="str">
+        <v>WB-BARASAT</v>
+      </c>
+      <c r="B7" t="str">
+        <v>Barasat</v>
+      </c>
+      <c r="C7" t="str">
+        <v>North 24 Parganas</v>
+      </c>
+      <c r="D7" t="str">
+        <v>West Bengal</v>
+      </c>
+      <c r="E7" t="str">
+        <v>19</v>
+      </c>
+      <c r="F7" t="str">
+        <v>India</v>
+      </c>
+      <c r="G7" t="str">
+        <v>Active</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="str">
+        <v>WB-BARDHAMAN</v>
+      </c>
+      <c r="B8" t="str">
+        <v>Bardhaman</v>
+      </c>
+      <c r="C8" t="str">
+        <v>Purba Bardhaman</v>
+      </c>
+      <c r="D8" t="str">
+        <v>West Bengal</v>
+      </c>
+      <c r="E8" t="str">
+        <v>19</v>
+      </c>
+      <c r="F8" t="str">
+        <v>India</v>
+      </c>
+      <c r="G8" t="str">
+        <v>Active</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="str">
+        <v>WB-BERHAMPORE</v>
+      </c>
+      <c r="B9" t="str">
+        <v>Berhampore</v>
+      </c>
+      <c r="C9" t="str">
+        <v>Murshidabad</v>
+      </c>
+      <c r="D9" t="str">
+        <v>West Bengal</v>
+      </c>
+      <c r="E9" t="str">
+        <v>19</v>
+      </c>
+      <c r="F9" t="str">
+        <v>India</v>
+      </c>
+      <c r="G9" t="str">
+        <v>Active</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="str">
+        <v>WB-BISHNUPUR</v>
+      </c>
+      <c r="B10" t="str">
+        <v>Bishnupur</v>
+      </c>
+      <c r="C10" t="str">
+        <v>Bankura</v>
+      </c>
+      <c r="D10" t="str">
+        <v>West Bengal</v>
+      </c>
+      <c r="E10" t="str">
+        <v>19</v>
+      </c>
+      <c r="F10" t="str">
+        <v>India</v>
+      </c>
+      <c r="G10" t="str">
+        <v>Active</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="str">
+        <v>WB-BOLPUR</v>
+      </c>
+      <c r="B11" t="str">
+        <v>Bolpur</v>
+      </c>
+      <c r="C11" t="str">
+        <v>Birbhum</v>
+      </c>
+      <c r="D11" t="str">
+        <v>West Bengal</v>
+      </c>
+      <c r="E11" t="str">
+        <v>19</v>
+      </c>
+      <c r="F11" t="str">
+        <v>India</v>
+      </c>
+      <c r="G11" t="str">
+        <v>Active</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="str">
+        <v>WB-COOCH-BEHAR</v>
+      </c>
+      <c r="B12" t="str">
+        <v>Cooch Behar</v>
+      </c>
+      <c r="C12" t="str">
+        <v>Cooch Behar</v>
+      </c>
+      <c r="D12" t="str">
+        <v>West Bengal</v>
+      </c>
+      <c r="E12" t="str">
+        <v>19</v>
+      </c>
+      <c r="F12" t="str">
+        <v>India</v>
+      </c>
+      <c r="G12" t="str">
+        <v>Active</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="str">
+        <v>WB-DARJEELING</v>
+      </c>
+      <c r="B13" t="str">
+        <v>Darjeeling</v>
+      </c>
+      <c r="C13" t="str">
+        <v>Darjeeling</v>
+      </c>
+      <c r="D13" t="str">
+        <v>West Bengal</v>
+      </c>
+      <c r="E13" t="str">
+        <v>19</v>
+      </c>
+      <c r="F13" t="str">
+        <v>India</v>
+      </c>
+      <c r="G13" t="str">
+        <v>Active</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="str">
+        <v>WB-DIGHA</v>
+      </c>
+      <c r="B14" t="str">
+        <v>Digha</v>
+      </c>
+      <c r="C14" t="str">
+        <v>Purba Medinipur</v>
+      </c>
+      <c r="D14" t="str">
+        <v>West Bengal</v>
+      </c>
+      <c r="E14" t="str">
+        <v>19</v>
+      </c>
+      <c r="F14" t="str">
+        <v>India</v>
+      </c>
+      <c r="G14" t="str">
+        <v>Active</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="str">
+        <v>WB-DURGAPUR</v>
+      </c>
+      <c r="B15" t="str">
+        <v>Durgapur</v>
+      </c>
+      <c r="C15" t="str">
+        <v>Paschim Bardhaman</v>
+      </c>
+      <c r="D15" t="str">
+        <v>West Bengal</v>
+      </c>
+      <c r="E15" t="str">
+        <v>19</v>
+      </c>
+      <c r="F15" t="str">
+        <v>India</v>
+      </c>
+      <c r="G15" t="str">
+        <v>Active</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="str">
+        <v>WB-ENGLISH-BAZAR</v>
+      </c>
+      <c r="B16" t="str">
+        <v>English Bazar</v>
+      </c>
+      <c r="C16" t="str">
+        <v>Malda</v>
+      </c>
+      <c r="D16" t="str">
+        <v>West Bengal</v>
+      </c>
+      <c r="E16" t="str">
+        <v>19</v>
+      </c>
+      <c r="F16" t="str">
+        <v>India</v>
+      </c>
+      <c r="G16" t="str">
+        <v>Active</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="str">
+        <v>WB-HALDIA</v>
+      </c>
+      <c r="B17" t="str">
+        <v>Haldia</v>
+      </c>
+      <c r="C17" t="str">
+        <v>Purba Medinipur</v>
+      </c>
+      <c r="D17" t="str">
+        <v>West Bengal</v>
+      </c>
+      <c r="E17" t="str">
+        <v>19</v>
+      </c>
+      <c r="F17" t="str">
+        <v>India</v>
+      </c>
+      <c r="G17" t="str">
+        <v>Active</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="str">
+        <v>WB-HOWRAH</v>
+      </c>
+      <c r="B18" t="str">
+        <v>Howrah</v>
+      </c>
+      <c r="C18" t="str">
+        <v>Howrah</v>
+      </c>
+      <c r="D18" t="str">
+        <v>West Bengal</v>
+      </c>
+      <c r="E18" t="str">
+        <v>19</v>
+      </c>
+      <c r="F18" t="str">
+        <v>India</v>
+      </c>
+      <c r="G18" t="str">
+        <v>Active</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="str">
+        <v>WB-JALPAIGURI</v>
+      </c>
+      <c r="B19" t="str">
+        <v>Jalpaiguri</v>
+      </c>
+      <c r="C19" t="str">
+        <v>Jalpaiguri</v>
+      </c>
+      <c r="D19" t="str">
+        <v>West Bengal</v>
+      </c>
+      <c r="E19" t="str">
+        <v>19</v>
+      </c>
+      <c r="F19" t="str">
+        <v>India</v>
+      </c>
+      <c r="G19" t="str">
+        <v>Active</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="str">
+        <v>WB-JHARGRAM</v>
+      </c>
+      <c r="B20" t="str">
+        <v>Jhargram</v>
+      </c>
+      <c r="C20" t="str">
+        <v>Jhargram</v>
+      </c>
+      <c r="D20" t="str">
+        <v>West Bengal</v>
+      </c>
+      <c r="E20" t="str">
+        <v>19</v>
+      </c>
+      <c r="F20" t="str">
+        <v>India</v>
+      </c>
+      <c r="G20" t="str">
+        <v>Active</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="str">
+        <v>WB-KALIMPONG</v>
+      </c>
+      <c r="B21" t="str">
+        <v>Kalimpong</v>
+      </c>
+      <c r="C21" t="str">
+        <v>Kalimpong</v>
+      </c>
+      <c r="D21" t="str">
+        <v>West Bengal</v>
+      </c>
+      <c r="E21" t="str">
+        <v>19</v>
+      </c>
+      <c r="F21" t="str">
+        <v>India</v>
+      </c>
+      <c r="G21" t="str">
+        <v>Active</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="str">
+        <v>WB-KALYANI</v>
+      </c>
+      <c r="B22" t="str">
+        <v>Kalyani</v>
+      </c>
+      <c r="C22" t="str">
+        <v>Nadia</v>
+      </c>
+      <c r="D22" t="str">
+        <v>West Bengal</v>
+      </c>
+      <c r="E22" t="str">
+        <v>19</v>
+      </c>
+      <c r="F22" t="str">
+        <v>India</v>
+      </c>
+      <c r="G22" t="str">
+        <v>Active</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="str">
+        <v>WB-KHARAGPUR</v>
+      </c>
+      <c r="B23" t="str">
+        <v>Kharagpur</v>
+      </c>
+      <c r="C23" t="str">
+        <v>Paschim Medinipur</v>
+      </c>
+      <c r="D23" t="str">
+        <v>West Bengal</v>
+      </c>
+      <c r="E23" t="str">
+        <v>19</v>
+      </c>
+      <c r="F23" t="str">
+        <v>India</v>
+      </c>
+      <c r="G23" t="str">
+        <v>Active</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="str">
+        <v>WB-KOLKATA</v>
+      </c>
+      <c r="B24" t="str">
+        <v>Kolkata</v>
+      </c>
+      <c r="C24" t="str">
+        <v>Kolkata</v>
+      </c>
+      <c r="D24" t="str">
+        <v>West Bengal</v>
+      </c>
+      <c r="E24" t="str">
+        <v>19</v>
+      </c>
+      <c r="F24" t="str">
+        <v>India</v>
+      </c>
+      <c r="G24" t="str">
+        <v>Active</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="str">
+        <v>WB-KRISHNANAGAR</v>
+      </c>
+      <c r="B25" t="str">
+        <v>Krishnanagar</v>
+      </c>
+      <c r="C25" t="str">
+        <v>Nadia</v>
+      </c>
+      <c r="D25" t="str">
+        <v>West Bengal</v>
+      </c>
+      <c r="E25" t="str">
+        <v>19</v>
+      </c>
+      <c r="F25" t="str">
+        <v>India</v>
+      </c>
+      <c r="G25" t="str">
+        <v>Active</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="str">
+        <v>WB-MALDA</v>
+      </c>
+      <c r="B26" t="str">
+        <v>Malda</v>
+      </c>
+      <c r="C26" t="str">
+        <v>Malda</v>
+      </c>
+      <c r="D26" t="str">
+        <v>West Bengal</v>
+      </c>
+      <c r="E26" t="str">
+        <v>19</v>
+      </c>
+      <c r="F26" t="str">
+        <v>India</v>
+      </c>
+      <c r="G26" t="str">
+        <v>Active</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="str">
+        <v>WB-MEDINIPUR</v>
+      </c>
+      <c r="B27" t="str">
+        <v>Medinipur</v>
+      </c>
+      <c r="C27" t="str">
+        <v>Paschim Medinipur</v>
+      </c>
+      <c r="D27" t="str">
+        <v>West Bengal</v>
+      </c>
+      <c r="E27" t="str">
+        <v>19</v>
+      </c>
+      <c r="F27" t="str">
+        <v>India</v>
+      </c>
+      <c r="G27" t="str">
+        <v>Active</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="str">
+        <v>WB-NEWTOWN</v>
+      </c>
+      <c r="B28" t="str">
+        <v>Newtown</v>
+      </c>
+      <c r="C28" t="str">
+        <v>North 24 Parganas</v>
+      </c>
+      <c r="D28" t="str">
+        <v>West Bengal</v>
+      </c>
+      <c r="E28" t="str">
+        <v>19</v>
+      </c>
+      <c r="F28" t="str">
+        <v>India</v>
+      </c>
+      <c r="G28" t="str">
+        <v>Active</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="str">
+        <v>WB-PURULIA</v>
+      </c>
+      <c r="B29" t="str">
+        <v>Purulia</v>
+      </c>
+      <c r="C29" t="str">
+        <v>Purulia</v>
+      </c>
+      <c r="D29" t="str">
+        <v>West Bengal</v>
+      </c>
+      <c r="E29" t="str">
+        <v>19</v>
+      </c>
+      <c r="F29" t="str">
+        <v>India</v>
+      </c>
+      <c r="G29" t="str">
+        <v>Active</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="str">
+        <v>WB-RAIGANJ</v>
+      </c>
+      <c r="B30" t="str">
+        <v>Raiganj</v>
+      </c>
+      <c r="C30" t="str">
+        <v>Uttar Dinajpur</v>
+      </c>
+      <c r="D30" t="str">
+        <v>West Bengal</v>
+      </c>
+      <c r="E30" t="str">
+        <v>19</v>
+      </c>
+      <c r="F30" t="str">
+        <v>India</v>
+      </c>
+      <c r="G30" t="str">
+        <v>Active</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="str">
+        <v>WB-RAJARHAT</v>
+      </c>
+      <c r="B31" t="str">
+        <v>Rajarhat</v>
+      </c>
+      <c r="C31" t="str">
+        <v>North 24 Parganas</v>
+      </c>
+      <c r="D31" t="str">
+        <v>West Bengal</v>
+      </c>
+      <c r="E31" t="str">
+        <v>19</v>
+      </c>
+      <c r="F31" t="str">
+        <v>India</v>
+      </c>
+      <c r="G31" t="str">
+        <v>Active</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="str">
+        <v>WB-RAMPURHAT</v>
+      </c>
+      <c r="B32" t="str">
+        <v>Rampurhat</v>
+      </c>
+      <c r="C32" t="str">
+        <v>Birbhum</v>
+      </c>
+      <c r="D32" t="str">
+        <v>West Bengal</v>
+      </c>
+      <c r="E32" t="str">
+        <v>19</v>
+      </c>
+      <c r="F32" t="str">
+        <v>India</v>
+      </c>
+      <c r="G32" t="str">
+        <v>Active</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="str">
+        <v>WB-SERAMPORE</v>
+      </c>
+      <c r="B33" t="str">
+        <v>Serampore</v>
+      </c>
+      <c r="C33" t="str">
+        <v>Hooghly</v>
+      </c>
+      <c r="D33" t="str">
+        <v>West Bengal</v>
+      </c>
+      <c r="E33" t="str">
+        <v>19</v>
+      </c>
+      <c r="F33" t="str">
+        <v>India</v>
+      </c>
+      <c r="G33" t="str">
+        <v>Active</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="str">
+        <v>WB-SILIGURI</v>
+      </c>
+      <c r="B34" t="str">
+        <v>Siliguri</v>
+      </c>
+      <c r="C34" t="str">
+        <v>Darjeeling</v>
+      </c>
+      <c r="D34" t="str">
+        <v>West Bengal</v>
+      </c>
+      <c r="E34" t="str">
+        <v>19</v>
+      </c>
+      <c r="F34" t="str">
+        <v>India</v>
+      </c>
+      <c r="G34" t="str">
+        <v>Active</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="str">
+        <v>WB-SURI</v>
+      </c>
+      <c r="B35" t="str">
+        <v>Suri</v>
+      </c>
+      <c r="C35" t="str">
+        <v>Birbhum</v>
+      </c>
+      <c r="D35" t="str">
+        <v>West Bengal</v>
+      </c>
+      <c r="E35" t="str">
+        <v>19</v>
+      </c>
+      <c r="F35" t="str">
+        <v>India</v>
+      </c>
+      <c r="G35" t="str">
+        <v>Active</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="str">
+        <v>WB-TAMLUK</v>
+      </c>
+      <c r="B36" t="str">
+        <v>Tamluk</v>
+      </c>
+      <c r="C36" t="str">
+        <v>Purba Medinipur</v>
+      </c>
+      <c r="D36" t="str">
+        <v>West Bengal</v>
+      </c>
+      <c r="E36" t="str">
+        <v>19</v>
+      </c>
+      <c r="F36" t="str">
+        <v>India</v>
+      </c>
+      <c r="G36" t="str">
+        <v>Active</v>
+      </c>
+    </row>
+  </sheetData>
+  <ignoredErrors>
+    <ignoredError numberStoredAsText="1" sqref="A1:G36"/>
+  </ignoredErrors>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Add HRMS country master default
</commit_message>
<xml_diff>
--- a/mock-db/hrms_mock_database.xlsx
+++ b/mock-db/hrms_mock_database.xlsx
@@ -12,6 +12,7 @@
     <sheet name="state_masters" sheetId="7" r:id="rId7"/>
     <sheet name="pincode_masters" sheetId="8" r:id="rId8"/>
     <sheet name="city_masters" sheetId="9" r:id="rId9"/>
+    <sheet name="country_masters" sheetId="10" r:id="rId10"/>
   </sheets>
 </workbook>
 </file>
@@ -437,6 +438,57 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:F2"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="str">
+        <v>country_code</v>
+      </c>
+      <c r="B1" t="str">
+        <v>country_name</v>
+      </c>
+      <c r="C1" t="str">
+        <v>iso2</v>
+      </c>
+      <c r="D1" t="str">
+        <v>phone_code</v>
+      </c>
+      <c r="E1" t="str">
+        <v>default_country</v>
+      </c>
+      <c r="F1" t="str">
+        <v>status</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="str">
+        <v>IN</v>
+      </c>
+      <c r="B2" t="str">
+        <v>India</v>
+      </c>
+      <c r="C2" t="str">
+        <v>IN</v>
+      </c>
+      <c r="D2" t="str">
+        <v>+91</v>
+      </c>
+      <c r="E2" t="str">
+        <v>TRUE</v>
+      </c>
+      <c r="F2" t="str">
+        <v>Active</v>
+      </c>
+    </row>
+  </sheetData>
+  <ignoredErrors>
+    <ignoredError numberStoredAsText="1" sqref="A1:F2"/>
+  </ignoredErrors>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:S1"/>

</xml_diff>

<commit_message>
Add HRMS primary entity onboarding
</commit_message>
<xml_diff>
--- a/mock-db/hrms_mock_database.xlsx
+++ b/mock-db/hrms_mock_database.xlsx
@@ -13,6 +13,7 @@
     <sheet name="pincode_masters" sheetId="8" r:id="rId8"/>
     <sheet name="city_masters" sheetId="9" r:id="rId9"/>
     <sheet name="country_masters" sheetId="10" r:id="rId10"/>
+    <sheet name="operating_contexts" sheetId="11" r:id="rId11"/>
   </sheets>
 </workbook>
 </file>
@@ -489,6 +490,40 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:G1"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="str">
+        <v>context_id</v>
+      </c>
+      <c r="B1" t="str">
+        <v>primary_entity_id</v>
+      </c>
+      <c r="C1" t="str">
+        <v>active_entity_id</v>
+      </c>
+      <c r="D1" t="str">
+        <v>entity_name</v>
+      </c>
+      <c r="E1" t="str">
+        <v>admin_name</v>
+      </c>
+      <c r="F1" t="str">
+        <v>admin_phone</v>
+      </c>
+      <c r="G1" t="str">
+        <v>status</v>
+      </c>
+    </row>
+  </sheetData>
+  <ignoredErrors>
+    <ignoredError numberStoredAsText="1" sqref="A1:G1"/>
+  </ignoredErrors>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:S1"/>

</xml_diff>

<commit_message>
Publish latest HRMS workflows
</commit_message>
<xml_diff>
--- a/mock-db/hrms_mock_database.xlsx
+++ b/mock-db/hrms_mock_database.xlsx
@@ -27,6 +27,7 @@
     <sheet name="attendance_incident_counters" sheetId="22" r:id="rId22"/>
     <sheet name="attendance_penalty_transactions" sheetId="23" r:id="rId23"/>
     <sheet name="attendance_penalty_audit" sheetId="24" r:id="rId24"/>
+    <sheet name="in_app_notifications" sheetId="25" r:id="rId25"/>
   </sheets>
 </workbook>
 </file>
@@ -590,23 +591,26 @@
 
 <file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:O1"/>
+  <dimension ref="A1:R1"/>
   <cols>
     <col min="1" max="1" width="12.83203125" customWidth="1"/>
     <col min="2" max="2" width="12.83203125" customWidth="1"/>
-    <col min="3" max="3" width="17.83203125" customWidth="1"/>
-    <col min="4" max="4" width="14.83203125" customWidth="1"/>
+    <col min="3" max="3" width="19.83203125" customWidth="1"/>
+    <col min="4" max="4" width="17.83203125" customWidth="1"/>
     <col min="5" max="5" width="14.83203125" customWidth="1"/>
     <col min="6" max="6" width="14.83203125" customWidth="1"/>
-    <col min="7" max="7" width="12.83203125" customWidth="1"/>
+    <col min="7" max="7" width="14.83203125" customWidth="1"/>
     <col min="8" max="8" width="12.83203125" customWidth="1"/>
-    <col min="9" max="9" width="13.83203125" customWidth="1"/>
-    <col min="10" max="10" width="14.83203125" customWidth="1"/>
-    <col min="11" max="11" width="13.83203125" customWidth="1"/>
-    <col min="12" max="12" width="15.83203125" customWidth="1"/>
-    <col min="13" max="13" width="12.83203125" customWidth="1"/>
-    <col min="14" max="14" width="12.83203125" customWidth="1"/>
-    <col min="15" max="15" width="12.83203125" customWidth="1"/>
+    <col min="9" max="9" width="12.83203125" customWidth="1"/>
+    <col min="10" max="10" width="13.83203125" customWidth="1"/>
+    <col min="11" max="11" width="12.83203125" customWidth="1"/>
+    <col min="12" max="12" width="14.83203125" customWidth="1"/>
+    <col min="13" max="13" width="14.83203125" customWidth="1"/>
+    <col min="14" max="14" width="13.83203125" customWidth="1"/>
+    <col min="15" max="15" width="15.83203125" customWidth="1"/>
+    <col min="16" max="16" width="12.83203125" customWidth="1"/>
+    <col min="17" max="17" width="12.83203125" customWidth="1"/>
+    <col min="18" max="18" width="12.83203125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -617,88 +621,98 @@
         <v>holiday_id</v>
       </c>
       <c r="C1" t="str">
+        <v>financial_year_id</v>
+      </c>
+      <c r="D1" t="str">
         <v>organization_id</v>
       </c>
-      <c r="D1" t="str">
+      <c r="E1" t="str">
         <v>holiday_date</v>
       </c>
-      <c r="E1" t="str">
+      <c r="F1" t="str">
         <v>holiday_name</v>
       </c>
-      <c r="F1" t="str">
+      <c r="G1" t="str">
         <v>holiday_type</v>
       </c>
-      <c r="G1" t="str">
+      <c r="H1" t="str">
         <v>scope_type</v>
       </c>
-      <c r="H1" t="str">
+      <c r="I1" t="str">
         <v>scope_key</v>
       </c>
-      <c r="I1" t="str">
+      <c r="J1" t="str">
         <v>scope_label</v>
       </c>
-      <c r="J1" t="str">
+      <c r="K1" t="str">
+        <v>scope_keys</v>
+      </c>
+      <c r="L1" t="str">
+        <v>scope_labels</v>
+      </c>
+      <c r="M1" t="str">
         <v>store_closed</v>
       </c>
-      <c r="K1" t="str">
+      <c r="N1" t="str">
         <v>co_eligible</v>
       </c>
-      <c r="L1" t="str">
+      <c r="O1" t="str">
         <v>calendar_year</v>
       </c>
-      <c r="M1" t="str">
+      <c r="P1" t="str">
         <v>status</v>
       </c>
-      <c r="N1" t="str">
+      <c r="Q1" t="str">
         <v>created_at</v>
       </c>
-      <c r="O1" t="str">
+      <c r="R1" t="str">
         <v>updated_at</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:O1"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:R1"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:AF1"/>
+  <dimension ref="A1:AG1"/>
   <cols>
     <col min="1" max="1" width="12.83203125" customWidth="1"/>
     <col min="2" max="2" width="12.83203125" customWidth="1"/>
-    <col min="3" max="3" width="13.83203125" customWidth="1"/>
-    <col min="4" max="4" width="15.83203125" customWidth="1"/>
-    <col min="5" max="5" width="17.83203125" customWidth="1"/>
-    <col min="6" max="6" width="13.83203125" customWidth="1"/>
-    <col min="7" max="7" width="12.83203125" customWidth="1"/>
+    <col min="3" max="3" width="19.83203125" customWidth="1"/>
+    <col min="4" max="4" width="13.83203125" customWidth="1"/>
+    <col min="5" max="5" width="15.83203125" customWidth="1"/>
+    <col min="6" max="6" width="17.83203125" customWidth="1"/>
+    <col min="7" max="7" width="13.83203125" customWidth="1"/>
     <col min="8" max="8" width="12.83203125" customWidth="1"/>
     <col min="9" max="9" width="12.83203125" customWidth="1"/>
     <col min="10" max="10" width="12.83203125" customWidth="1"/>
-    <col min="11" max="11" width="17.83203125" customWidth="1"/>
-    <col min="12" max="12" width="14.83203125" customWidth="1"/>
-    <col min="13" max="13" width="12.83203125" customWidth="1"/>
-    <col min="14" max="14" width="15.83203125" customWidth="1"/>
-    <col min="15" max="15" width="14.83203125" customWidth="1"/>
-    <col min="16" max="16" width="16.83203125" customWidth="1"/>
-    <col min="17" max="17" width="18.83203125" customWidth="1"/>
-    <col min="18" max="18" width="12.83203125" customWidth="1"/>
+    <col min="11" max="11" width="12.83203125" customWidth="1"/>
+    <col min="12" max="12" width="17.83203125" customWidth="1"/>
+    <col min="13" max="13" width="14.83203125" customWidth="1"/>
+    <col min="14" max="14" width="12.83203125" customWidth="1"/>
+    <col min="15" max="15" width="15.83203125" customWidth="1"/>
+    <col min="16" max="16" width="14.83203125" customWidth="1"/>
+    <col min="17" max="17" width="16.83203125" customWidth="1"/>
+    <col min="18" max="18" width="18.83203125" customWidth="1"/>
     <col min="19" max="19" width="12.83203125" customWidth="1"/>
-    <col min="20" max="20" width="13.83203125" customWidth="1"/>
-    <col min="21" max="21" width="12.83203125" customWidth="1"/>
+    <col min="20" max="20" width="12.83203125" customWidth="1"/>
+    <col min="21" max="21" width="13.83203125" customWidth="1"/>
     <col min="22" max="22" width="12.83203125" customWidth="1"/>
     <col min="23" max="23" width="12.83203125" customWidth="1"/>
-    <col min="24" max="24" width="15.83203125" customWidth="1"/>
-    <col min="25" max="25" width="17.83203125" customWidth="1"/>
-    <col min="26" max="26" width="16.83203125" customWidth="1"/>
+    <col min="24" max="24" width="12.83203125" customWidth="1"/>
+    <col min="25" max="25" width="15.83203125" customWidth="1"/>
+    <col min="26" max="26" width="17.83203125" customWidth="1"/>
     <col min="27" max="27" width="16.83203125" customWidth="1"/>
-    <col min="28" max="28" width="20.83203125" customWidth="1"/>
-    <col min="29" max="29" width="19.83203125" customWidth="1"/>
-    <col min="30" max="30" width="12.83203125" customWidth="1"/>
+    <col min="28" max="28" width="16.83203125" customWidth="1"/>
+    <col min="29" max="29" width="20.83203125" customWidth="1"/>
+    <col min="30" max="30" width="19.83203125" customWidth="1"/>
     <col min="31" max="31" width="12.83203125" customWidth="1"/>
     <col min="32" max="32" width="12.83203125" customWidth="1"/>
+    <col min="33" max="33" width="12.83203125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -709,99 +723,102 @@
         <v>ledger_id</v>
       </c>
       <c r="C1" t="str">
+        <v>financial_year_id</v>
+      </c>
+      <c r="D1" t="str">
         <v>employee_id</v>
       </c>
-      <c r="D1" t="str">
+      <c r="E1" t="str">
         <v>employee_name</v>
       </c>
-      <c r="E1" t="str">
+      <c r="F1" t="str">
         <v>organization_id</v>
       </c>
-      <c r="F1" t="str">
+      <c r="G1" t="str">
         <v>location_id</v>
       </c>
-      <c r="G1" t="str">
+      <c r="H1" t="str">
         <v>location</v>
       </c>
-      <c r="H1" t="str">
+      <c r="I1" t="str">
         <v>policy_id</v>
       </c>
-      <c r="I1" t="str">
+      <c r="J1" t="str">
         <v>leave_code</v>
       </c>
-      <c r="J1" t="str">
+      <c r="K1" t="str">
         <v>leave_name</v>
       </c>
-      <c r="K1" t="str">
+      <c r="L1" t="str">
         <v>opening_balance</v>
       </c>
-      <c r="L1" t="str">
+      <c r="M1" t="str">
         <v>accrued_days</v>
       </c>
-      <c r="M1" t="str">
+      <c r="N1" t="str">
         <v>used_days</v>
       </c>
-      <c r="N1" t="str">
+      <c r="O1" t="str">
         <v>adjusted_days</v>
       </c>
-      <c r="O1" t="str">
+      <c r="P1" t="str">
         <v>pending_days</v>
       </c>
-      <c r="P1" t="str">
+      <c r="Q1" t="str">
         <v>available_days</v>
       </c>
-      <c r="Q1" t="str">
+      <c r="R1" t="str">
         <v>transaction_date</v>
       </c>
-      <c r="R1" t="str">
+      <c r="S1" t="str">
         <v>as_of_date</v>
       </c>
-      <c r="S1" t="str">
+      <c r="T1" t="str">
         <v>status</v>
       </c>
-      <c r="T1" t="str">
+      <c r="U1" t="str">
         <v>source_type</v>
       </c>
-      <c r="U1" t="str">
+      <c r="V1" t="str">
         <v>source_id</v>
       </c>
-      <c r="V1" t="str">
+      <c r="W1" t="str">
         <v>holiday_id</v>
       </c>
-      <c r="W1" t="str">
+      <c r="X1" t="str">
         <v>units</v>
       </c>
-      <c r="X1" t="str">
+      <c r="Y1" t="str">
         <v>pay_treatment</v>
       </c>
-      <c r="Y1" t="str">
+      <c r="Z1" t="str">
         <v>workflow_status</v>
       </c>
-      <c r="Z1" t="str">
+      <c r="AA1" t="str">
         <v>payroll_period</v>
       </c>
-      <c r="AA1" t="str">
+      <c r="AB1" t="str">
         <v>payroll_status</v>
       </c>
-      <c r="AB1" t="str">
+      <c r="AC1" t="str">
         <v>payroll_applied_at</v>
       </c>
-      <c r="AC1" t="str">
+      <c r="AD1" t="str">
         <v>reversed_entry_id</v>
       </c>
-      <c r="AD1" t="str">
+      <c r="AE1" t="str">
         <v>created_at</v>
       </c>
-      <c r="AE1" t="str">
+      <c r="AF1" t="str">
         <v>updated_at</v>
       </c>
-      <c r="AF1" t="str">
+      <c r="AG1" t="str">
         <v>history</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:AF1"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:AG1"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -1230,28 +1247,29 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:T1"/>
+  <dimension ref="A1:U1"/>
   <cols>
     <col min="1" max="1" width="12.83203125" customWidth="1"/>
     <col min="2" max="2" width="12.83203125" customWidth="1"/>
-    <col min="3" max="3" width="13.83203125" customWidth="1"/>
-    <col min="4" max="4" width="12.83203125" customWidth="1"/>
+    <col min="3" max="3" width="19.83203125" customWidth="1"/>
+    <col min="4" max="4" width="13.83203125" customWidth="1"/>
     <col min="5" max="5" width="12.83203125" customWidth="1"/>
     <col min="6" max="6" width="12.83203125" customWidth="1"/>
-    <col min="7" max="7" width="13.83203125" customWidth="1"/>
-    <col min="8" max="8" width="12.83203125" customWidth="1"/>
+    <col min="7" max="7" width="12.83203125" customWidth="1"/>
+    <col min="8" max="8" width="13.83203125" customWidth="1"/>
     <col min="9" max="9" width="12.83203125" customWidth="1"/>
     <col min="10" max="10" width="12.83203125" customWidth="1"/>
     <col min="11" max="11" width="12.83203125" customWidth="1"/>
     <col min="12" max="12" width="12.83203125" customWidth="1"/>
-    <col min="13" max="13" width="16.83203125" customWidth="1"/>
-    <col min="14" max="14" width="12.83203125" customWidth="1"/>
+    <col min="13" max="13" width="12.83203125" customWidth="1"/>
+    <col min="14" max="14" width="16.83203125" customWidth="1"/>
     <col min="15" max="15" width="12.83203125" customWidth="1"/>
     <col min="16" max="16" width="12.83203125" customWidth="1"/>
     <col min="17" max="17" width="12.83203125" customWidth="1"/>
     <col min="18" max="18" width="12.83203125" customWidth="1"/>
-    <col min="19" max="19" width="18.83203125" customWidth="1"/>
-    <col min="20" max="20" width="12.83203125" customWidth="1"/>
+    <col min="19" max="19" width="12.83203125" customWidth="1"/>
+    <col min="20" max="20" width="18.83203125" customWidth="1"/>
+    <col min="21" max="21" width="12.83203125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1262,63 +1280,66 @@
         <v>id</v>
       </c>
       <c r="C1" t="str">
+        <v>financial_year_id</v>
+      </c>
+      <c r="D1" t="str">
         <v>employee_id</v>
       </c>
-      <c r="D1" t="str">
+      <c r="E1" t="str">
         <v>name</v>
       </c>
-      <c r="E1" t="str">
+      <c r="F1" t="str">
         <v>initials</v>
       </c>
-      <c r="F1" t="str">
+      <c r="G1" t="str">
         <v>entity_id</v>
       </c>
-      <c r="G1" t="str">
+      <c r="H1" t="str">
         <v>location_id</v>
       </c>
-      <c r="H1" t="str">
+      <c r="I1" t="str">
         <v>location</v>
       </c>
-      <c r="I1" t="str">
+      <c r="J1" t="str">
         <v>work_date</v>
       </c>
-      <c r="J1" t="str">
+      <c r="K1" t="str">
         <v>shift</v>
       </c>
-      <c r="K1" t="str">
+      <c r="L1" t="str">
         <v>checkIn</v>
       </c>
-      <c r="L1" t="str">
+      <c r="M1" t="str">
         <v>checkOut</v>
       </c>
-      <c r="M1" t="str">
+      <c r="N1" t="str">
         <v>worked_minutes</v>
       </c>
-      <c r="N1" t="str">
+      <c r="O1" t="str">
         <v>issue</v>
       </c>
-      <c r="O1" t="str">
+      <c r="P1" t="str">
         <v>status</v>
       </c>
-      <c r="P1" t="str">
+      <c r="Q1" t="str">
         <v>source</v>
       </c>
-      <c r="Q1" t="str">
+      <c r="R1" t="str">
         <v>roster_id</v>
       </c>
-      <c r="R1" t="str">
+      <c r="S1" t="str">
         <v>source_id</v>
       </c>
-      <c r="S1" t="str">
+      <c r="T1" t="str">
         <v>leave_request_id</v>
       </c>
-      <c r="T1" t="str">
+      <c r="U1" t="str">
         <v>policy_id</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:T1"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:U1"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -1499,178 +1520,186 @@
 
 <file path=xl/worksheets/sheet22.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:N1"/>
+  <dimension ref="A1:O1"/>
   <cols>
     <col min="1" max="1" width="12.83203125" customWidth="1"/>
     <col min="2" max="2" width="12.83203125" customWidth="1"/>
-    <col min="3" max="3" width="12.83203125" customWidth="1"/>
+    <col min="3" max="3" width="19.83203125" customWidth="1"/>
     <col min="4" max="4" width="12.83203125" customWidth="1"/>
-    <col min="5" max="5" width="13.83203125" customWidth="1"/>
-    <col min="6" max="6" width="12.83203125" customWidth="1"/>
+    <col min="5" max="5" width="12.83203125" customWidth="1"/>
+    <col min="6" max="6" width="13.83203125" customWidth="1"/>
+    <col min="7" max="7" width="12.83203125" customWidth="1"/>
+    <col min="8" max="8" width="15.83203125" customWidth="1"/>
+    <col min="9" max="9" width="18.83203125" customWidth="1"/>
+    <col min="10" max="10" width="16.83203125" customWidth="1"/>
+    <col min="11" max="11" width="27.83203125" customWidth="1"/>
+    <col min="12" max="12" width="12.83203125" customWidth="1"/>
+    <col min="13" max="13" width="20.83203125" customWidth="1"/>
+    <col min="14" max="14" width="12.83203125" customWidth="1"/>
+    <col min="15" max="15" width="12.83203125" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="str">
+        <v>tenant_id</v>
+      </c>
+      <c r="B1" t="str">
+        <v>counter_id</v>
+      </c>
+      <c r="C1" t="str">
+        <v>financial_year_id</v>
+      </c>
+      <c r="D1" t="str">
+        <v>rule_id</v>
+      </c>
+      <c r="E1" t="str">
+        <v>policy_id</v>
+      </c>
+      <c r="F1" t="str">
+        <v>employee_id</v>
+      </c>
+      <c r="G1" t="str">
+        <v>period_key</v>
+      </c>
+      <c r="H1" t="str">
+        <v>incident_code</v>
+      </c>
+      <c r="I1" t="str">
+        <v>occurrence_count</v>
+      </c>
+      <c r="J1" t="str">
+        <v>consumed_count</v>
+      </c>
+      <c r="K1" t="str">
+        <v>qualifying_attendance_ids</v>
+      </c>
+      <c r="L1" t="str">
+        <v>status</v>
+      </c>
+      <c r="M1" t="str">
+        <v>last_incident_date</v>
+      </c>
+      <c r="N1" t="str">
+        <v>created_at</v>
+      </c>
+      <c r="O1" t="str">
+        <v>updated_at</v>
+      </c>
+    </row>
+  </sheetData>
+  <ignoredErrors>
+    <ignoredError numberStoredAsText="1" sqref="A1:O1"/>
+  </ignoredErrors>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet23.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:X1"/>
+  <cols>
+    <col min="1" max="1" width="12.83203125" customWidth="1"/>
+    <col min="2" max="2" width="16.83203125" customWidth="1"/>
+    <col min="3" max="3" width="19.83203125" customWidth="1"/>
+    <col min="4" max="4" width="12.83203125" customWidth="1"/>
+    <col min="5" max="5" width="12.83203125" customWidth="1"/>
+    <col min="6" max="6" width="13.83203125" customWidth="1"/>
     <col min="7" max="7" width="15.83203125" customWidth="1"/>
-    <col min="8" max="8" width="18.83203125" customWidth="1"/>
-    <col min="9" max="9" width="16.83203125" customWidth="1"/>
-    <col min="10" max="10" width="27.83203125" customWidth="1"/>
-    <col min="11" max="11" width="12.83203125" customWidth="1"/>
-    <col min="12" max="12" width="20.83203125" customWidth="1"/>
-    <col min="13" max="13" width="12.83203125" customWidth="1"/>
-    <col min="14" max="14" width="12.83203125" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" t="str">
-        <v>tenant_id</v>
-      </c>
-      <c r="B1" t="str">
-        <v>counter_id</v>
-      </c>
-      <c r="C1" t="str">
+    <col min="8" max="8" width="12.83203125" customWidth="1"/>
+    <col min="9" max="9" width="13.83203125" customWidth="1"/>
+    <col min="10" max="10" width="12.83203125" customWidth="1"/>
+    <col min="11" max="11" width="15.83203125" customWidth="1"/>
+    <col min="12" max="12" width="22.83203125" customWidth="1"/>
+    <col min="13" max="13" width="23.83203125" customWidth="1"/>
+    <col min="14" max="14" width="14.83203125" customWidth="1"/>
+    <col min="15" max="15" width="18.83203125" customWidth="1"/>
+    <col min="16" max="16" width="12.83203125" customWidth="1"/>
+    <col min="17" max="17" width="12.83203125" customWidth="1"/>
+    <col min="18" max="18" width="17.83203125" customWidth="1"/>
+    <col min="19" max="19" width="17.83203125" customWidth="1"/>
+    <col min="20" max="20" width="12.83203125" customWidth="1"/>
+    <col min="21" max="21" width="17.83203125" customWidth="1"/>
+    <col min="22" max="22" width="13.83203125" customWidth="1"/>
+    <col min="23" max="23" width="12.83203125" customWidth="1"/>
+    <col min="24" max="24" width="12.83203125" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="str">
+        <v>tenant_id</v>
+      </c>
+      <c r="B1" t="str">
+        <v>transaction_id</v>
+      </c>
+      <c r="C1" t="str">
+        <v>financial_year_id</v>
+      </c>
+      <c r="D1" t="str">
         <v>rule_id</v>
       </c>
-      <c r="D1" t="str">
+      <c r="E1" t="str">
         <v>policy_id</v>
       </c>
-      <c r="E1" t="str">
+      <c r="F1" t="str">
         <v>employee_id</v>
       </c>
-      <c r="F1" t="str">
+      <c r="G1" t="str">
+        <v>employee_name</v>
+      </c>
+      <c r="H1" t="str">
+        <v>entity_id</v>
+      </c>
+      <c r="I1" t="str">
+        <v>location_id</v>
+      </c>
+      <c r="J1" t="str">
         <v>period_key</v>
       </c>
-      <c r="G1" t="str">
+      <c r="K1" t="str">
         <v>incident_code</v>
       </c>
-      <c r="H1" t="str">
-        <v>occurrence_count</v>
-      </c>
-      <c r="I1" t="str">
-        <v>consumed_count</v>
-      </c>
-      <c r="J1" t="str">
-        <v>qualifying_attendance_ids</v>
-      </c>
-      <c r="K1" t="str">
-        <v>status</v>
-      </c>
       <c r="L1" t="str">
-        <v>last_incident_date</v>
+        <v>occurrence_threshold</v>
       </c>
       <c r="M1" t="str">
+        <v>source_attendance_ids</v>
+      </c>
+      <c r="N1" t="str">
+        <v>source_dates</v>
+      </c>
+      <c r="O1" t="str">
+        <v>consequence_type</v>
+      </c>
+      <c r="P1" t="str">
+        <v>leave_code</v>
+      </c>
+      <c r="Q1" t="str">
+        <v>units</v>
+      </c>
+      <c r="R1" t="str">
+        <v>fallback_action</v>
+      </c>
+      <c r="S1" t="str">
+        <v>workflow_status</v>
+      </c>
+      <c r="T1" t="str">
+        <v>ledger_id</v>
+      </c>
+      <c r="U1" t="str">
+        <v>reversal_reason</v>
+      </c>
+      <c r="V1" t="str">
+        <v>reversed_at</v>
+      </c>
+      <c r="W1" t="str">
         <v>created_at</v>
       </c>
-      <c r="N1" t="str">
+      <c r="X1" t="str">
         <v>updated_at</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:N1"/>
-  </ignoredErrors>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet23.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:W1"/>
-  <cols>
-    <col min="1" max="1" width="12.83203125" customWidth="1"/>
-    <col min="2" max="2" width="16.83203125" customWidth="1"/>
-    <col min="3" max="3" width="12.83203125" customWidth="1"/>
-    <col min="4" max="4" width="12.83203125" customWidth="1"/>
-    <col min="5" max="5" width="13.83203125" customWidth="1"/>
-    <col min="6" max="6" width="15.83203125" customWidth="1"/>
-    <col min="7" max="7" width="12.83203125" customWidth="1"/>
-    <col min="8" max="8" width="13.83203125" customWidth="1"/>
-    <col min="9" max="9" width="12.83203125" customWidth="1"/>
-    <col min="10" max="10" width="15.83203125" customWidth="1"/>
-    <col min="11" max="11" width="22.83203125" customWidth="1"/>
-    <col min="12" max="12" width="23.83203125" customWidth="1"/>
-    <col min="13" max="13" width="14.83203125" customWidth="1"/>
-    <col min="14" max="14" width="18.83203125" customWidth="1"/>
-    <col min="15" max="15" width="12.83203125" customWidth="1"/>
-    <col min="16" max="16" width="12.83203125" customWidth="1"/>
-    <col min="17" max="17" width="17.83203125" customWidth="1"/>
-    <col min="18" max="18" width="17.83203125" customWidth="1"/>
-    <col min="19" max="19" width="12.83203125" customWidth="1"/>
-    <col min="20" max="20" width="17.83203125" customWidth="1"/>
-    <col min="21" max="21" width="13.83203125" customWidth="1"/>
-    <col min="22" max="22" width="12.83203125" customWidth="1"/>
-    <col min="23" max="23" width="12.83203125" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" t="str">
-        <v>tenant_id</v>
-      </c>
-      <c r="B1" t="str">
-        <v>transaction_id</v>
-      </c>
-      <c r="C1" t="str">
-        <v>rule_id</v>
-      </c>
-      <c r="D1" t="str">
-        <v>policy_id</v>
-      </c>
-      <c r="E1" t="str">
-        <v>employee_id</v>
-      </c>
-      <c r="F1" t="str">
-        <v>employee_name</v>
-      </c>
-      <c r="G1" t="str">
-        <v>entity_id</v>
-      </c>
-      <c r="H1" t="str">
-        <v>location_id</v>
-      </c>
-      <c r="I1" t="str">
-        <v>period_key</v>
-      </c>
-      <c r="J1" t="str">
-        <v>incident_code</v>
-      </c>
-      <c r="K1" t="str">
-        <v>occurrence_threshold</v>
-      </c>
-      <c r="L1" t="str">
-        <v>source_attendance_ids</v>
-      </c>
-      <c r="M1" t="str">
-        <v>source_dates</v>
-      </c>
-      <c r="N1" t="str">
-        <v>consequence_type</v>
-      </c>
-      <c r="O1" t="str">
-        <v>leave_code</v>
-      </c>
-      <c r="P1" t="str">
-        <v>units</v>
-      </c>
-      <c r="Q1" t="str">
-        <v>fallback_action</v>
-      </c>
-      <c r="R1" t="str">
-        <v>workflow_status</v>
-      </c>
-      <c r="S1" t="str">
-        <v>ledger_id</v>
-      </c>
-      <c r="T1" t="str">
-        <v>reversal_reason</v>
-      </c>
-      <c r="U1" t="str">
-        <v>reversed_at</v>
-      </c>
-      <c r="V1" t="str">
-        <v>created_at</v>
-      </c>
-      <c r="W1" t="str">
-        <v>updated_at</v>
-      </c>
-    </row>
-  </sheetData>
-  <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:W1"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:X1"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -1726,6 +1755,117 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet25.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:X1"/>
+  <cols>
+    <col min="1" max="1" width="12.83203125" customWidth="1"/>
+    <col min="2" max="2" width="17.83203125" customWidth="1"/>
+    <col min="3" max="3" width="13.83203125" customWidth="1"/>
+    <col min="4" max="4" width="12.83203125" customWidth="1"/>
+    <col min="5" max="5" width="16.83203125" customWidth="1"/>
+    <col min="6" max="6" width="23.83203125" customWidth="1"/>
+    <col min="7" max="7" width="15.83203125" customWidth="1"/>
+    <col min="8" max="8" width="12.83203125" customWidth="1"/>
+    <col min="9" max="9" width="13.83203125" customWidth="1"/>
+    <col min="10" max="10" width="12.83203125" customWidth="1"/>
+    <col min="11" max="11" width="12.83203125" customWidth="1"/>
+    <col min="12" max="12" width="12.83203125" customWidth="1"/>
+    <col min="13" max="13" width="12.83203125" customWidth="1"/>
+    <col min="14" max="14" width="13.83203125" customWidth="1"/>
+    <col min="15" max="15" width="13.83203125" customWidth="1"/>
+    <col min="16" max="16" width="12.83203125" customWidth="1"/>
+    <col min="17" max="17" width="15.83203125" customWidth="1"/>
+    <col min="18" max="18" width="22.83203125" customWidth="1"/>
+    <col min="19" max="19" width="14.83203125" customWidth="1"/>
+    <col min="20" max="20" width="12.83203125" customWidth="1"/>
+    <col min="21" max="21" width="12.83203125" customWidth="1"/>
+    <col min="22" max="22" width="12.83203125" customWidth="1"/>
+    <col min="23" max="23" width="12.83203125" customWidth="1"/>
+    <col min="24" max="24" width="13.83203125" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="str">
+        <v>tenant_id</v>
+      </c>
+      <c r="B1" t="str">
+        <v>notification_id</v>
+      </c>
+      <c r="C1" t="str">
+        <v>source_type</v>
+      </c>
+      <c r="D1" t="str">
+        <v>source_id</v>
+      </c>
+      <c r="E1" t="str">
+        <v>recipient_type</v>
+      </c>
+      <c r="F1" t="str">
+        <v>recipient_employee_id</v>
+      </c>
+      <c r="G1" t="str">
+        <v>employee_name</v>
+      </c>
+      <c r="H1" t="str">
+        <v>entity_id</v>
+      </c>
+      <c r="I1" t="str">
+        <v>location_id</v>
+      </c>
+      <c r="J1" t="str">
+        <v>title</v>
+      </c>
+      <c r="K1" t="str">
+        <v>message</v>
+      </c>
+      <c r="L1" t="str">
+        <v>severity</v>
+      </c>
+      <c r="M1" t="str">
+        <v>status</v>
+      </c>
+      <c r="N1" t="str">
+        <v>read_status</v>
+      </c>
+      <c r="O1" t="str">
+        <v>action_page</v>
+      </c>
+      <c r="P1" t="str">
+        <v>period_key</v>
+      </c>
+      <c r="Q1" t="str">
+        <v>incident_code</v>
+      </c>
+      <c r="R1" t="str">
+        <v>occurrence_threshold</v>
+      </c>
+      <c r="S1" t="str">
+        <v>source_dates</v>
+      </c>
+      <c r="T1" t="str">
+        <v>payload</v>
+      </c>
+      <c r="U1" t="str">
+        <v>created_at</v>
+      </c>
+      <c r="V1" t="str">
+        <v>updated_at</v>
+      </c>
+      <c r="W1" t="str">
+        <v>read_at</v>
+      </c>
+      <c r="X1" t="str">
+        <v>resolved_at</v>
+      </c>
+    </row>
+  </sheetData>
+  <ignoredErrors>
+    <ignoredError numberStoredAsText="1" sqref="A1:X1"/>
+  </ignoredErrors>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:F1"/>
@@ -1767,12 +1907,12 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:AD1"/>
+  <dimension ref="A1:AE1"/>
   <cols>
     <col min="1" max="1" width="12.83203125" customWidth="1"/>
     <col min="2" max="2" width="12.83203125" customWidth="1"/>
-    <col min="3" max="3" width="13.83203125" customWidth="1"/>
-    <col min="4" max="4" width="12.83203125" customWidth="1"/>
+    <col min="3" max="3" width="19.83203125" customWidth="1"/>
+    <col min="4" max="4" width="13.83203125" customWidth="1"/>
     <col min="5" max="5" width="12.83203125" customWidth="1"/>
     <col min="6" max="6" width="12.83203125" customWidth="1"/>
     <col min="7" max="7" width="12.83203125" customWidth="1"/>
@@ -1783,22 +1923,23 @@
     <col min="12" max="12" width="12.83203125" customWidth="1"/>
     <col min="13" max="13" width="12.83203125" customWidth="1"/>
     <col min="14" max="14" width="12.83203125" customWidth="1"/>
-    <col min="15" max="15" width="16.83203125" customWidth="1"/>
-    <col min="16" max="16" width="13.83203125" customWidth="1"/>
+    <col min="15" max="15" width="12.83203125" customWidth="1"/>
+    <col min="16" max="16" width="16.83203125" customWidth="1"/>
     <col min="17" max="17" width="13.83203125" customWidth="1"/>
-    <col min="18" max="18" width="19.83203125" customWidth="1"/>
-    <col min="19" max="19" width="23.83203125" customWidth="1"/>
-    <col min="20" max="20" width="27.83203125" customWidth="1"/>
-    <col min="21" max="21" width="12.83203125" customWidth="1"/>
-    <col min="22" max="22" width="21.83203125" customWidth="1"/>
-    <col min="23" max="23" width="12.83203125" customWidth="1"/>
-    <col min="24" max="24" width="16.83203125" customWidth="1"/>
-    <col min="25" max="25" width="15.83203125" customWidth="1"/>
-    <col min="26" max="26" width="17.83203125" customWidth="1"/>
-    <col min="27" max="27" width="28.83203125" customWidth="1"/>
-    <col min="28" max="28" width="18.83203125" customWidth="1"/>
-    <col min="29" max="29" width="12.83203125" customWidth="1"/>
+    <col min="18" max="18" width="13.83203125" customWidth="1"/>
+    <col min="19" max="19" width="19.83203125" customWidth="1"/>
+    <col min="20" max="20" width="23.83203125" customWidth="1"/>
+    <col min="21" max="21" width="27.83203125" customWidth="1"/>
+    <col min="22" max="22" width="12.83203125" customWidth="1"/>
+    <col min="23" max="23" width="21.83203125" customWidth="1"/>
+    <col min="24" max="24" width="12.83203125" customWidth="1"/>
+    <col min="25" max="25" width="16.83203125" customWidth="1"/>
+    <col min="26" max="26" width="15.83203125" customWidth="1"/>
+    <col min="27" max="27" width="17.83203125" customWidth="1"/>
+    <col min="28" max="28" width="28.83203125" customWidth="1"/>
+    <col min="29" max="29" width="18.83203125" customWidth="1"/>
     <col min="30" max="30" width="12.83203125" customWidth="1"/>
+    <col min="31" max="31" width="12.83203125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1809,93 +1950,96 @@
         <v>roster_id</v>
       </c>
       <c r="C1" t="str">
+        <v>financial_year_id</v>
+      </c>
+      <c r="D1" t="str">
         <v>location_id</v>
       </c>
-      <c r="D1" t="str">
+      <c r="E1" t="str">
         <v>period</v>
       </c>
-      <c r="E1" t="str">
+      <c r="F1" t="str">
         <v>start_date</v>
       </c>
-      <c r="F1" t="str">
+      <c r="G1" t="str">
         <v>end_date</v>
       </c>
-      <c r="G1" t="str">
+      <c r="H1" t="str">
         <v>version</v>
       </c>
-      <c r="H1" t="str">
+      <c r="I1" t="str">
         <v>status</v>
       </c>
-      <c r="I1" t="str">
+      <c r="J1" t="str">
         <v>filled</v>
       </c>
-      <c r="J1" t="str">
+      <c r="K1" t="str">
         <v>open</v>
       </c>
-      <c r="K1" t="str">
+      <c r="L1" t="str">
         <v>conflicts</v>
       </c>
-      <c r="L1" t="str">
+      <c r="M1" t="str">
         <v>keyholder</v>
       </c>
-      <c r="M1" t="str">
+      <c r="N1" t="str">
         <v>updated</v>
       </c>
-      <c r="N1" t="str">
+      <c r="O1" t="str">
         <v>issue</v>
       </c>
-      <c r="O1" t="str">
+      <c r="P1" t="str">
         <v>leave_handling</v>
       </c>
-      <c r="P1" t="str">
+      <c r="Q1" t="str">
         <v>assignments</v>
       </c>
-      <c r="Q1" t="str">
+      <c r="R1" t="str">
         <v>weekly_offs</v>
       </c>
-      <c r="R1" t="str">
+      <c r="S1" t="str">
         <v>draft_weekly_offs</v>
       </c>
-      <c r="S1" t="str">
+      <c r="T1" t="str">
         <v>weekly_off_allowances</v>
       </c>
-      <c r="T1" t="str">
+      <c r="U1" t="str">
         <v>weekly_off_baseline_ready</v>
       </c>
-      <c r="U1" t="str">
+      <c r="V1" t="str">
         <v>leave_days</v>
       </c>
-      <c r="V1" t="str">
+      <c r="W1" t="str">
         <v>rotation_exceptions</v>
       </c>
-      <c r="W1" t="str">
+      <c r="X1" t="str">
         <v>open_slots</v>
       </c>
-      <c r="X1" t="str">
+      <c r="Y1" t="str">
         <v>conflicts_list</v>
       </c>
-      <c r="Y1" t="str">
+      <c r="Z1" t="str">
         <v>warnings_list</v>
       </c>
-      <c r="Z1" t="str">
+      <c r="AA1" t="str">
         <v>override_reason</v>
       </c>
-      <c r="AA1" t="str">
+      <c r="AB1" t="str">
         <v>override_warning_signature</v>
       </c>
-      <c r="AB1" t="str">
+      <c r="AC1" t="str">
         <v>comp_off_entries</v>
       </c>
-      <c r="AC1" t="str">
+      <c r="AD1" t="str">
         <v>excluded</v>
       </c>
-      <c r="AD1" t="str">
+      <c r="AE1" t="str">
         <v>history</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:AD1"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:AE1"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -1949,29 +2093,30 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:U1"/>
+  <dimension ref="A1:V1"/>
   <cols>
     <col min="1" max="1" width="12.83203125" customWidth="1"/>
     <col min="2" max="2" width="12.83203125" customWidth="1"/>
-    <col min="3" max="3" width="12.83203125" customWidth="1"/>
+    <col min="3" max="3" width="19.83203125" customWidth="1"/>
     <col min="4" max="4" width="12.83203125" customWidth="1"/>
     <col min="5" max="5" width="12.83203125" customWidth="1"/>
     <col min="6" max="6" width="12.83203125" customWidth="1"/>
     <col min="7" max="7" width="12.83203125" customWidth="1"/>
-    <col min="8" max="8" width="14.83203125" customWidth="1"/>
-    <col min="9" max="9" width="12.83203125" customWidth="1"/>
-    <col min="10" max="10" width="16.83203125" customWidth="1"/>
-    <col min="11" max="11" width="12.83203125" customWidth="1"/>
-    <col min="12" max="12" width="15.83203125" customWidth="1"/>
-    <col min="13" max="13" width="13.83203125" customWidth="1"/>
-    <col min="14" max="14" width="19.83203125" customWidth="1"/>
-    <col min="15" max="15" width="18.83203125" customWidth="1"/>
-    <col min="16" max="16" width="12.83203125" customWidth="1"/>
-    <col min="17" max="17" width="13.83203125" customWidth="1"/>
-    <col min="18" max="18" width="14.83203125" customWidth="1"/>
-    <col min="19" max="19" width="12.83203125" customWidth="1"/>
+    <col min="8" max="8" width="12.83203125" customWidth="1"/>
+    <col min="9" max="9" width="14.83203125" customWidth="1"/>
+    <col min="10" max="10" width="12.83203125" customWidth="1"/>
+    <col min="11" max="11" width="16.83203125" customWidth="1"/>
+    <col min="12" max="12" width="12.83203125" customWidth="1"/>
+    <col min="13" max="13" width="15.83203125" customWidth="1"/>
+    <col min="14" max="14" width="13.83203125" customWidth="1"/>
+    <col min="15" max="15" width="19.83203125" customWidth="1"/>
+    <col min="16" max="16" width="18.83203125" customWidth="1"/>
+    <col min="17" max="17" width="12.83203125" customWidth="1"/>
+    <col min="18" max="18" width="13.83203125" customWidth="1"/>
+    <col min="19" max="19" width="14.83203125" customWidth="1"/>
     <col min="20" max="20" width="12.83203125" customWidth="1"/>
     <col min="21" max="21" width="12.83203125" customWidth="1"/>
+    <col min="22" max="22" width="12.83203125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1982,85 +2127,89 @@
         <v>row_id</v>
       </c>
       <c r="C1" t="str">
+        <v>financial_year_id</v>
+      </c>
+      <c r="D1" t="str">
         <v>pageKey</v>
       </c>
-      <c r="D1" t="str">
+      <c r="E1" t="str">
         <v>role_id</v>
       </c>
-      <c r="E1" t="str">
+      <c r="F1" t="str">
         <v>role_code</v>
       </c>
-      <c r="F1" t="str">
+      <c r="G1" t="str">
         <v>role_name</v>
       </c>
-      <c r="G1" t="str">
+      <c r="H1" t="str">
         <v>name</v>
       </c>
-      <c r="H1" t="str">
+      <c r="I1" t="str">
         <v>module_scope</v>
       </c>
-      <c r="I1" t="str">
+      <c r="J1" t="str">
         <v>scope</v>
       </c>
-      <c r="J1" t="str">
+      <c r="K1" t="str">
         <v>entity_context</v>
       </c>
-      <c r="K1" t="str">
+      <c r="L1" t="str">
         <v>data_scope</v>
       </c>
-      <c r="L1" t="str">
+      <c r="M1" t="str">
         <v>location_rule</v>
       </c>
-      <c r="M1" t="str">
+      <c r="N1" t="str">
         <v>permissions</v>
       </c>
-      <c r="N1" t="str">
+      <c r="O1" t="str">
         <v>permission_matrix</v>
       </c>
-      <c r="O1" t="str">
+      <c r="P1" t="str">
         <v>permission_codes</v>
       </c>
-      <c r="P1" t="str">
+      <c r="Q1" t="str">
         <v>users</v>
       </c>
-      <c r="Q1" t="str">
+      <c r="R1" t="str">
         <v>lastChanged</v>
       </c>
-      <c r="R1" t="str">
+      <c r="S1" t="str">
         <v>last_changed</v>
       </c>
-      <c r="S1" t="str">
+      <c r="T1" t="str">
         <v>status</v>
       </c>
-      <c r="T1" t="str">
+      <c r="U1" t="str">
         <v>details</v>
       </c>
-      <c r="U1" t="str">
+      <c r="V1" t="str">
         <v>cells</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:U1"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:V1"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:K1"/>
+  <dimension ref="A1:L1"/>
   <cols>
     <col min="1" max="1" width="12.83203125" customWidth="1"/>
     <col min="2" max="2" width="12.83203125" customWidth="1"/>
-    <col min="3" max="3" width="12.83203125" customWidth="1"/>
-    <col min="4" max="4" width="13.83203125" customWidth="1"/>
+    <col min="3" max="3" width="19.83203125" customWidth="1"/>
+    <col min="4" max="4" width="12.83203125" customWidth="1"/>
     <col min="5" max="5" width="13.83203125" customWidth="1"/>
-    <col min="6" max="6" width="12.83203125" customWidth="1"/>
+    <col min="6" max="6" width="13.83203125" customWidth="1"/>
     <col min="7" max="7" width="12.83203125" customWidth="1"/>
     <col min="8" max="8" width="12.83203125" customWidth="1"/>
     <col min="9" max="9" width="12.83203125" customWidth="1"/>
     <col min="10" max="10" width="12.83203125" customWidth="1"/>
     <col min="11" max="11" width="12.83203125" customWidth="1"/>
+    <col min="12" max="12" width="12.83203125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -2071,36 +2220,39 @@
         <v>policy_id</v>
       </c>
       <c r="C1" t="str">
+        <v>financial_year_id</v>
+      </c>
+      <c r="D1" t="str">
         <v>entity_id</v>
       </c>
-      <c r="D1" t="str">
+      <c r="E1" t="str">
         <v>policy_code</v>
       </c>
-      <c r="E1" t="str">
+      <c r="F1" t="str">
         <v>policy_name</v>
       </c>
-      <c r="F1" t="str">
+      <c r="G1" t="str">
         <v>status</v>
       </c>
-      <c r="G1" t="str">
+      <c r="H1" t="str">
         <v>version</v>
       </c>
-      <c r="H1" t="str">
+      <c r="I1" t="str">
         <v>rules</v>
       </c>
-      <c r="I1" t="str">
+      <c r="J1" t="str">
         <v>history</v>
       </c>
-      <c r="J1" t="str">
+      <c r="K1" t="str">
         <v>created_at</v>
       </c>
-      <c r="K1" t="str">
+      <c r="L1" t="str">
         <v>updated_at</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:K1"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:L1"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -2158,18 +2310,19 @@
 
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:J1"/>
+  <dimension ref="A1:K1"/>
   <cols>
     <col min="1" max="1" width="12.83203125" customWidth="1"/>
     <col min="2" max="2" width="12.83203125" customWidth="1"/>
-    <col min="3" max="3" width="17.83203125" customWidth="1"/>
-    <col min="4" max="4" width="13.83203125" customWidth="1"/>
+    <col min="3" max="3" width="19.83203125" customWidth="1"/>
+    <col min="4" max="4" width="17.83203125" customWidth="1"/>
     <col min="5" max="5" width="13.83203125" customWidth="1"/>
-    <col min="6" max="6" width="12.83203125" customWidth="1"/>
+    <col min="6" max="6" width="13.83203125" customWidth="1"/>
     <col min="7" max="7" width="12.83203125" customWidth="1"/>
     <col min="8" max="8" width="12.83203125" customWidth="1"/>
     <col min="9" max="9" width="12.83203125" customWidth="1"/>
     <col min="10" max="10" width="12.83203125" customWidth="1"/>
+    <col min="11" max="11" width="12.83203125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -2180,33 +2333,36 @@
         <v>policy_id</v>
       </c>
       <c r="C1" t="str">
+        <v>financial_year_id</v>
+      </c>
+      <c r="D1" t="str">
         <v>organization_id</v>
       </c>
-      <c r="D1" t="str">
+      <c r="E1" t="str">
         <v>policy_code</v>
       </c>
-      <c r="E1" t="str">
+      <c r="F1" t="str">
         <v>policy_name</v>
       </c>
-      <c r="F1" t="str">
+      <c r="G1" t="str">
         <v>status</v>
       </c>
-      <c r="G1" t="str">
+      <c r="H1" t="str">
         <v>version</v>
       </c>
-      <c r="H1" t="str">
+      <c r="I1" t="str">
         <v>history</v>
       </c>
-      <c r="I1" t="str">
+      <c r="J1" t="str">
         <v>created_at</v>
       </c>
-      <c r="J1" t="str">
+      <c r="K1" t="str">
         <v>updated_at</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:J1"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:K1"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>